<commit_message>
Add data table, equations and updated README
</commit_message>
<xml_diff>
--- a/data/dictionaries/T4_CP1_data_start.xlsx
+++ b/data/dictionaries/T4_CP1_data_start.xlsx
@@ -12,6 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Dictionary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gene_Label_Dictionary" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Split_Dictionary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Table" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gene_Table_Example" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,8 +35,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -51,6 +56,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3B5C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -64,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -73,6 +83,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -440,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -454,56 +468,63 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>What this is: the 'start-evidence package' for the data part of Checkpoint 1 (download log + source, gene/label and split dictionaries).</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>GitHub repository: https://github.com/JacksonMahr782/Machine-Learning</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Status: all 6 sources accessed and downloaded (Oct 15-19, 2026). Proof screenshots are in proof/.</t>
+          <t>What this is: the 'start-evidence package' for the data part of Checkpoint 1 (download log + source, gene/label and split dictionaries).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Step 1: open each URL in 'Download_Log', note the release/version shown on the page, start the download, screenshot it.</t>
+          <t>Status: all 6 sources accessed and downloaded (Oct 15-19, 2026). Proof screenshots are in proof/.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Step 2: fill in date, size and status (Done / In progress / Not started). Unfinished big downloads are OK at Checkpoint 1.</t>
+          <t>Step 1: open each URL in 'Download_Log', note the release/version shown on the page, start the download, screenshot it.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Step 3: the three dictionary sheets are drafts of what the tables WILL contain. Check them as a group; no data has to be computed yet.</t>
+          <t>Step 2: fill in date, size and status (Done / In progress / Not started). Unfinished big downloads are OK at Checkpoint 1.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Key rule (leakage): nothing derived from DepMap gene effects may be used as a feature. DepMap only makes the label.</t>
+          <t>Step 3: the three dictionary sheets are drafts of what the tables WILL contain. Check them as a group; no data has to be computed yet.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Key rule (scope): the TROP2 paper reproduction (E-MTAB-16585) and the LUAD dependency model are two separate tasks.</t>
+          <t>Key rule (leakage): nothing derived from DepMap gene effects may be used as a feature. DepMap only makes the label.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Key rule (scope): the TROP2 paper reproduction (E-MTAB-16585) and the LUAD dependency model are two separate tasks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Release versions were read from each site's page by Jackson on the download date; see the Download_Log.</t>
         </is>
@@ -634,7 +655,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Downloaded (bulk zip failed first; re-downloaded). Check which of the 12 .txt files each zip holds before Checkpoint 2 (owner: Jackson)</t>
+          <t>Done: all 12 processed .txt files confirmed present (checked by Jackson, 2026-10-21). Next: load with Figure_01.ipynb</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -1748,4 +1769,891 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Release / version</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Size (as shown in Windows)</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Date downloaded</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>One row is</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>One column is</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Used for</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CRISPRGeneEffect.csv</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>DepMap Portal</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Public 26Q3</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>485,489 KB (~474 MB)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>One cell line (ModelID)</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>One gene ('SYMBOL (ENTREZ)')</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Label only (Chronos effect)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Model.csv</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>DepMap Portal</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Public 26Q3</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>772 KB</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>One cell line</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>One attribute (ModelID, OncotreeCode, lineage...)</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Picking LUAD lines (OncotreeCode = LUAD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>TCGA-LUAD.star_tpm.tsv.gz</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>UCSC Xena (GDC TCGA-LUAD hub)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>star_tpm version not recorded</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>TSV (gzip)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>164,516 KB (~161 MB)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>One gene (Ensembl ID)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>One sample (tumour or normal)</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Features: expression, enrichment, variability</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>TCGA-LUAD.clinical.tsv.gz</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>UCSC Xena (GDC TCGA-LUAD hub)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>phenotype v09-07-2024</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>TSV (gzip)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>147 KB</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>One sample</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>One clinical/phenotype field</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Tumour vs normal sample type</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>luad_tcga_pan_can_atlas_2018.tar.gz (data_cna.txt inside)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>cBioPortal</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>TCGA LUAD PanCancer Atlas 2018</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>TAR.GZ (tab-separated text inside)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>912,219 KB (~891 MB)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>One gene (Hugo_Symbol)</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>One tumour sample (GISTIC -2, -1, 0, +1, +2)</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Features: amplification frequency</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>subcellular_location.tsv.zip</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Human Protein Atlas</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Ensembl 109</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>TSV (zip)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>247 KB</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>One gene</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Gene, Main/Additional location, Reliability</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Surface eligibility + split stratification</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>E-MTAB-16585.zip</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ArrayExpress (TROP2 paper)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>E-MTAB-16585</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>ZIP of processed .txt files</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>1,304,207 KB</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>(12 processed .txt files across the 3 zips)</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>(cells x genes + cell metadata)</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Paper reproduction (Figure 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>E-MTAB-16585-2.zip</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ArrayExpress (TROP2 paper)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>E-MTAB-16585</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>ZIP of processed .txt files</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>1,281,957 KB</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>(see row 7)</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>(see row 7)</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Paper reproduction (Figure 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>E-MTAB-16585 3.zip</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>ArrayExpress (TROP2 paper)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>E-MTAB-16585</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>ZIP of processed .txt files</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>1,076,004 KB</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>(see row 7)</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>(see row 7)</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Paper reproduction (Figure 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>figures/Figure_01.ipynb</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>GitHub ORCA-HD/TROP2_in_CRC</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>commit d04c1bd (2026-07-01)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Jupyter notebook</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>592 KB</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 (viewed)</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Paper reproduction code</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>gene_symbol</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>expr_mean_tumor</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>expr_enrichment</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>expr_sd_tumor</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>gistic_amp_freq</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>gistic_highamp_freq</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>is_surface</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>n_luad_lines</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>label_dependency</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>GENE_A</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>0.18</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>0.03</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>0.42</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>train</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>GENE_B</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>-0.5</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>GENE_C</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>8.7</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>0.31</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>0.07</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>GENE_D</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>(unlabeled)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Example values only, not real data. Shows the column layout of the Checkpoint 2 gene table.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>